<commit_message>
Update deliverables spreadsheet: Tasks 16+17 added, Task 16 marked complete
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ZMspc4a6jeX4r9dJ8VaYm
</commit_message>
<xml_diff>
--- a/DVM_Fire_Division_Deliverables.xlsx
+++ b/DVM_Fire_Division_Deliverables.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Deliverables" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Project Tasks" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,47 +26,41 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="13"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="005A6E82"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
+      <name val="Segoe UI"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
+      <b val="1"/>
       <color rgb="001C2B3A"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
+      <color rgb="001C2B3A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="001E6B42"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="005A6E82"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -85,17 +79,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4F6FA"/>
+        <fgColor rgb="00DDE3EC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003D5A80"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -105,7 +94,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -140,43 +129,36 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -544,297 +526,347 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DVM Fire Division — UtilizeCore Deliverables</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
+          <t>DVM Fire Division — UtilizeCore Project Tracker   |   Go-Live: August 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Go-Live Date: August 1, 2026</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Last Updated: July 13, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="6" customHeight="1">
-      <c r="A3" s="4" t="n"/>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+          <t>Last Updated: 2026-07-14   |   Total: 17   |   Complete: 8   |   Pending: 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Due</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="6" t="n">
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Companywide filter template for FLS (work orders only)</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Get clients from Silpa</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
+          <t>Service Call and Maintenance customers only</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Get sites from Anthony</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="8" t="inlineStr"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Get clients from Silpa</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>Silpa</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Create scheduled services for all quarterly services</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr"/>
-      <c r="F6" s="12" t="inlineStr"/>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Get sites from Anthony</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Anthony Pasquarella</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Add DVM Fire's rates</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="8" t="inlineStr"/>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Create scheduled services for all quarterly services</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr"/>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Track inventory</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr"/>
-      <c r="F8" s="12" t="inlineStr"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Add DVM Fire's rates</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr"/>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Track employee hours</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="8" t="inlineStr"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Track inventory</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr"/>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Separate WOs for PTO/Holiday/Sick; regular hours via UC check-in &amp; check-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Create a dummy reactive work order to show Silpa</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr"/>
-      <c r="F10" s="12" t="inlineStr"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Track employee hours</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr"/>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Demo/training reactive WO for Silpa review</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Create a dummy PM work order for Silpa</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Separate WOs for PTO, Holiday, Sick; regular hours via UC check-in &amp; check-out</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Create a dummy reactive work order to show Silpa</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>Silpa</t>
-        </is>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Preventive Maintenance WO demo for Silpa</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Reach out to Frank Trotta</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Find out what UC dashboards &amp; reports he uses to track payroll</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Build New Services and Tasks</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Assign Department to Service and Tasks</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Assign Trades and Services to Sites</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>Demo/training reactive WO</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="inlineStr"/>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Create a dummy PM work order for Silpa</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Silpa</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Match Building Reports to Work Order Reports</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>Preventive Maintenance WO demo</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr"/>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Reach out to Frank Trotta re: payroll dashboards</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>Frank Trotta</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr"/>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Create all clients in UC</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>Find out what UC dashboards &amp; reports he uses to track payroll</t>
-        </is>
-      </c>
-      <c r="F14" s="12" t="inlineStr"/>
+      <c r="D18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Create all sites</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr"/>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Add Accumatica Customer ID's</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:C2"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark Task 17 complete: Add Accumatica Customer IDs
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ZMspc4a6jeX4r9dJ8VaYm
</commit_message>
<xml_diff>
--- a/DVM_Fire_Division_Deliverables.xlsx
+++ b/DVM_Fire_Division_Deliverables.xlsx
@@ -545,7 +545,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last Updated: 2026-07-14   |   Total: 17   |   Complete: 8   |   Pending: 9</t>
+          <t>Last Updated: 2026-07-15   |   Total: 17   |   Complete: 9   |   Pending: 8</t>
         </is>
       </c>
     </row>
@@ -856,9 +856,9 @@
           <t>Add Accumatica Customer ID's</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr"/>

</xml_diff>

<commit_message>
Mark Tasks 6 & 13 in progress: working with Anthony
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ZMspc4a6jeX4r9dJ8VaYm
</commit_message>
<xml_diff>
--- a/DVM_Fire_Division_Deliverables.xlsx
+++ b/DVM_Fire_Division_Deliverables.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,8 +59,14 @@
       <color rgb="005A6E82"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="009B5E08"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -100,6 +106,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EDF0F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -129,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -159,6 +170,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -545,7 +559,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last Updated: 2026-07-15   |   Total: 17   |   Complete: 9   |   Pending: 8</t>
+          <t>Last Updated: 2026-07-15   |   Total: 17   |   Complete: 9   |   In Progress: 2   |   Pending: 6</t>
         </is>
       </c>
     </row>
@@ -664,12 +678,16 @@
           <t>Track inventory</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr"/>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Working with Anthony</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="5" t="n">
@@ -792,12 +810,16 @@
           <t>Assign Trades and Services to Sites</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr"/>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Working with Anthony</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="8" t="n">

</xml_diff>